<commit_message>
Update soil moisture calibration workbook and local tool permissions
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/soil_moisture_calibration_curve.xlsx
+++ b/soil_moisture_calibration_curve.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/581c023685c7c5b8/Documents/GitHub/ai-farm/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="74" documentId="8_{65C0100A-4DE8-4BA5-98B4-D9C23DC27DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{72F5F255-0EE7-4825-B987-F3891ECACA06}"/>
+  <xr:revisionPtr revIDLastSave="79" documentId="8_{65C0100A-4DE8-4BA5-98B4-D9C23DC27DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD4695F3-FC74-434A-BEC1-DBF35E03E719}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{337DBDA1-1B73-4EA8-9F24-E0B0878FC1B2}"/>
   </bookViews>
   <sheets>
-    <sheet name="工作表1" sheetId="1" r:id="rId1"/>
+    <sheet name="calibration" sheetId="1" r:id="rId1"/>
+    <sheet name="test" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -108,10 +109,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -431,7 +428,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDFA2D17-5B94-4A9E-AB4F-034D488D0DC5}">
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.125" bestFit="1" customWidth="1"/>
@@ -518,10 +515,21 @@
         <v>55.99</v>
       </c>
     </row>
-    <row r="17" spans="12:12" x14ac:dyDescent="0.25">
-      <c r="L17">
-        <f>EXP(-0.00258653*250+4.91733458)</f>
-        <v>71.571867160371667</v>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3E18DF4-9ADD-4227-BB0A-7FA9A0D7B4B1}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1">
+        <f>EXP(-0.00258653*288+4.91733458)</f>
+        <v>64.871860029582578</v>
       </c>
     </row>
   </sheetData>

</xml_diff>